<commit_message>
Move mailing data (PDF templates, sent-letter history) to Supabase
- pipeline_db.py now reads/writes pdf_templates and letters_sent via the
  Supabase REST API instead of local SQLite, using SUPABASE_URL and
  SUPABASE_SECRET_KEY from the environment. Same function signatures as
  before, so dashboard.py needed no changes.
- Added supabase_schema.sql (the table DDL, run manually once via the
  Supabase SQL Editor since the REST API can't execute DDL).
- Existing local data (pdf template + all sent-letter history) migrated
  over and verified to match.
- Dropped the Zip column from the confirmed-leads table display (still
  used for address validation, sending, and CSV export) and made the
  stats cards stretch full page width - both to reduce visual crowding.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/UT/uta/2026-07-27.xlsx
+++ b/UT/uta/2026-07-27.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,6 +476,11 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
+          <t>Posted Date</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
           <t>Property Value</t>
         </is>
       </c>
@@ -516,6 +521,11 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>No address on file</t>
         </is>
       </c>
@@ -566,6 +576,11 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
           <t>$420,900</t>
         </is>
       </c>
@@ -616,7 +631,758 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
           <t>$631,500</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Steven Verl Smith</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SMITH, BRAD STEVEN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>40:342:0006</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>636 W 250 NORTH</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>LINDON</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>84042</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>brad</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/us/obituaries/name/steven-smith-obituary?id=62047873</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>$886,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Steven Verl Smith</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>SMITH, DEREK STEVEN</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>66:442:0409</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2128 E 100 NORTH</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>SPANISH FORK</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>84660</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>derek</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/us/obituaries/name/steven-smith-obituary?id=62047873</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>$587,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Steven Verl Smith</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>SMITH, JOSHUA STEVEN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>08:140:0012</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>261 W 500 SOUTH</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>PAYSON</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>84651</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>joshua</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/us/obituaries/name/steven-smith-obituary?id=62047873</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>$444,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Grace Elaine Guymon Jones</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>JONES, GRACE E</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>26:018:0004</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>674 CANYON RD</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>SPRINGVILLE</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>84663</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>initial E matches deceased's own name 'Elaine'</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>$604,200</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Grace Elaine Guymon Jones</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>JONES, GRACE E</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>48:025:0003</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1501 E 1500 NORTH</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>PROVO</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>84604</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>initial E matches deceased's own name 'Elaine'</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>$810,900</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Haley Fox</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>FOX, HALEY MICHELLE</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>45:634:0018</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>462 S SUNLAND WAY</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SARATOGA SPRINGS</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>84045</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>michelle</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/us/obituaries/richfieldreaper/name/haley-fox-obituary?id=62035499</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>$417,100</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Max A Jensen</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>JENSEN, MAX A</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>43:231:0001</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>1975 N 300 WEST</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>MAPLETON</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>84664</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>initial A matches deceased's own name 'A'</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>$728,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Robert J Petersen</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>PETERSEN, ROBERT J</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>05:038:0013</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>156 E 400 NORTH</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>PROVO</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>84606</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'J'</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/person/robert-j-petersen-61935201</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>$703,800</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Robert J Petersen</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>PETERSEN, ROBERT J</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>05:077:0013</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>658 N 400 EAST</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>PROVO</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>84606</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'J'</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/person/robert-j-petersen-61935201</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>$1,018,400</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Robert J Petersen</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>PETERSEN, ROBERT J</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>36:032:0006</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>10 N 700 EAST</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>OREM</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>84097</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'J'</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/person/robert-j-petersen-61935201</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>$496,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Robert J Petersen</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>PETERSEN, ROBERT J</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>42:006:0022</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2880 CHIPPEWA WY</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>PROVO</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>84604</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'J'</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://www.legacy.com/person/robert-j-petersen-61935201</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>$769,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Virginia Elizabeth Temple</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>TEMPLE, VIRGINIA E</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>46:449:0006</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>211 N 1140 EAST</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>PAYSON</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>84651</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>initial E matches deceased's own name 'Elizabeth'</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>$316,600</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>John Earl Burningham</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>BURNINGHAM, JOHN E</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>46:147:0023</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>1058 W 1100 NORTH</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>PROVO</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>84604</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>initial E matches deceased's own name 'Earl'</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>$450,300</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Marsha Johnson Steggell</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>STEGGELL, MARSHA J</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>46:097:0045</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>587 S 1500 EAST</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>SPANISH FORK</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>UT</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>84660</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>initial J matches deceased's own name 'Johnson'</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>2026-07-27</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>$401,100</t>
         </is>
       </c>
     </row>

</xml_diff>